<commit_message>
test(hw03): execute GUI checklist and capture defect evidence
</commit_message>
<xml_diff>
--- a/docs/assignments/HW03/deliverables/checklist/gui_checklist.xlsx
+++ b/docs/assignments/HW03/deliverables/checklist/gui_checklist.xlsx
@@ -454,7 +454,7 @@
     <col width="11" customWidth="1" min="9" max="9"/>
     <col width="42" customWidth="1" min="10" max="10"/>
     <col width="42" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="42" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -552,12 +552,12 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Table displays correctly with formatted currency ₫</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>Cart rendered 5 columns (Sản phẩm, Giá, Số lượng, Thành tiền, Thao tác) and displayed the formatted total.</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -572,7 +572,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
+          <t>Executed twice on Google Chrome 151 / Windows.</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr"/>
@@ -610,12 +610,12 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>First click only increments internal clickCount state; item is not added until second click</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>After one click on Product Detail, the cart remained empty; a second click is required.</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -630,10 +630,14 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr"/>
+          <t>Executed twice on Google Chrome 151 / Windows. First click does not add the product.</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>bugs/evidence_images/bug_001_first_click_cart_empty.png</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -668,12 +672,12 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>System accepts 0 and negative quantities without error validation</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>The product was added with quantity -5 and a negative subtotal (iPhone 15 Pro Max 30.000.000 ₫ -5 -150.000.000 ₫ Xóa).</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -688,10 +692,14 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr"/>
+          <t>Executed twice on Google Chrome 151 / Windows. No minimum or validation feedback is provided.</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>bugs/evidence_images/bug_002_negative_quantity.png</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -726,12 +734,12 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>parseInt('2.5', 10) truncates input to integer 2 silently without notifying user</t>
-        </is>
-      </c>
-      <c r="H5" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>Entering 2.5 produced cart quantity 2 without any validation message.</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -746,10 +754,14 @@
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr"/>
+          <t>Executed twice on Google Chrome 151 / Windows. The decimal was silently truncated by parseInt().</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>bugs/evidence_images/bug_003_decimal_quantity_truncated.png</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -784,12 +796,12 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Total amount is rendered inside an editable &lt;input type='number'&gt;, allowing manual price alteration</t>
-        </is>
-      </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>Checkout total is rendered in an editable number input and accepted manual changes.</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -804,10 +816,14 @@
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr"/>
+          <t>Executed twice on Google Chrome 151 / Windows. The displayed/payment total is client-editable.</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>bugs/evidence_images/bug_006_editable_checkout_total.png</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -842,12 +858,12 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Both buttons navigate to correct routes smoothly</t>
-        </is>
-      </c>
-      <c r="H7" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>Continue shopping links to the product list and the checkout control is available.</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -862,7 +878,7 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
+          <t>Executed twice on Google Chrome 151 / Windows.</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr"/>
@@ -900,12 +916,12 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Triggers alert 'Bạn cần đăng nhập để thanh toán!' and redirects to /login</t>
-        </is>
-      </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>Unauthenticated checkout displayed “Bạn cần đăng nhập để thanh toán!” and redirected to /login.</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -920,7 +936,7 @@
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
+          <t>Executed twice on Google Chrome 151 / Windows.</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr"/>
@@ -958,12 +974,12 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Displays empty cart message and CTA link</t>
-        </is>
-      </c>
-      <c r="H9" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>The empty-cart message and continue-shopping link were displayed after removing the item.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -978,7 +994,7 @@
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
+          <t>Executed twice on Google Chrome 151 / Windows.</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr"/>
@@ -1016,12 +1032,12 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Cart state remains populated in CartContext and header badge after payment</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>The purchased item remained in the cart after checkout completed.</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -1036,10 +1052,14 @@
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr"/>
+          <t>Executed twice on Google Chrome 151 / Windows. Checkout does not invoke clearCart().</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>bugs/evidence_images/bug_007_cart_retained_after_checkout.png</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1074,7 +1094,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Items and total sum displayed cleanly on mobile layout</t>
+          <t>Not executed on a qualifying mobile environment.</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
@@ -1094,7 +1114,7 @@
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
+          <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr"/>
@@ -1132,7 +1152,7 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Code executes parsed + 1, so typing 2 results in quantity 3</t>
+          <t>Not executed on a qualifying mobile environment.</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
@@ -1142,7 +1162,7 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>BUG-009</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1152,7 +1172,7 @@
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
+          <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr"/>
@@ -1190,7 +1210,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Payload executes cart.slice(0, -1), dropping the last item from checkout order payload</t>
+          <t>Not executed on a qualifying mobile environment.</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
@@ -1200,7 +1220,7 @@
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>BUG-008</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
@@ -1210,7 +1230,7 @@
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
+          <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr"/>
@@ -1248,7 +1268,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Item removed immediately and total recalculated</t>
+          <t>Not executed on a qualifying mobile environment.</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
@@ -1268,7 +1288,7 @@
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
+          <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr"/>
@@ -1306,12 +1326,12 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Displays 'Chờ xác nhận' yellow badge</t>
-        </is>
-      </c>
-      <c r="H15" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>A newly created order displayed “Chờ xác nhận” with the pending badge style.</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -1326,7 +1346,7 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
+          <t>Executed twice on Google Chrome 151 / Windows.</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr"/>
@@ -1364,12 +1384,12 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Status updates through pending -&gt; confirmed -&gt; shipping -&gt; delivered</t>
-        </is>
-      </c>
-      <c r="H16" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>The API accepted the valid sequence confirmed → shipping → delivered.</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1384,7 +1404,7 @@
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
+          <t>Executed twice on Google Chrome 151 / Windows.</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr"/>
@@ -1422,12 +1442,12 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Backend and Web UI permit user to cancel order in shipping state</t>
-        </is>
-      </c>
-      <c r="H17" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>The cancellation request returned HTTP 200; the shipping order became canceled.</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -1442,10 +1462,14 @@
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
-        </is>
-      </c>
-      <c r="L17" s="2" t="inlineStr"/>
+          <t>Executed twice on Google Chrome 151 / Windows. Shipping is incorrectly treated as cancelable.</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>bugs/evidence_images/bug_010_shipping_order_canceled.png</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1480,12 +1504,12 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Backend allows transition and Admin UI renders active 'Đánh dấu Đã giao' button</t>
-        </is>
-      </c>
-      <c r="H18" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>Canceled → delivered returned HTTP 200; the admin UI displayed the resulting delivered state.</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -1500,10 +1524,14 @@
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
-        </is>
-      </c>
-      <c r="L18" s="2" t="inlineStr"/>
+          <t>Executed twice on Google Chrome 151 / Windows. A terminal canceled order can escape to delivered.</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>bugs/evidence_images/bug_011_canceled_order_delivered.png</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1538,17 +1566,17 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Coupon applied successfully with price reduction</t>
-        </is>
-      </c>
-      <c r="H19" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>SAVE10 (10%) reported savings of -270,000,000 ₫ and a final total of 300,000,000 ₫; the correct values are 3,000,000 ₫ and 27,000,000 ₫.</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>BUG-015</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -1558,10 +1586,14 @@
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
-        </is>
-      </c>
-      <c r="L19" s="2" t="inlineStr"/>
+          <t>Executed twice on Google Chrome 151 / Windows. Percentage discount calculation is incorrect.</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>bugs/evidence_images/bug_015_percent_coupon_calculation.png</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1596,12 +1628,12 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Displays clear invalid coupon error message</t>
-        </is>
-      </c>
-      <c r="H20" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>The invalid coupon displayed the inline message “Mã giảm giá không tồn tại hoặc đã bị vô hiệu hóa”.</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -1616,7 +1648,7 @@
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
+          <t>Executed twice on Google Chrome 151 / Windows.</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr"/>
@@ -1654,12 +1686,12 @@
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>Successfully navigates to Profile order tab</t>
-        </is>
-      </c>
-      <c r="H21" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>Checkout displayed a dedicated success state and provided navigation back to the home page.</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
@@ -1674,7 +1706,7 @@
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
+          <t>Executed twice on Google Chrome 151 / Windows.</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr"/>
@@ -1712,12 +1744,12 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>No further state changes allowed on delivered orders</t>
-        </is>
-      </c>
-      <c r="H22" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>A delivered order rejected a transition back to confirmed with HTTP 400.</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -1732,7 +1764,7 @@
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
+          <t>Executed twice on Google Chrome 151 / Windows.</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr"/>
@@ -1770,12 +1802,12 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Layout renders cleanly on desktop screens</t>
-        </is>
-      </c>
-      <c r="H23" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>Order history rendered as a structured five-column table at 1440×1000.</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -1790,7 +1822,7 @@
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
+          <t>Executed twice on Google Chrome 151 / Windows.</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr"/>
@@ -1828,12 +1860,12 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Badges correctly styled with distinct colors</t>
-        </is>
-      </c>
-      <c r="H24" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>Status badges rendered localized labels: Đã hủy, Đã giao, Chờ xác nhận, Chờ xác nhận.</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -1848,7 +1880,7 @@
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
+          <t>Executed twice on Google Chrome 151 / Windows.</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr"/>
@@ -1886,12 +1918,12 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Validation regex /^[1-9][0-9]{8,9}$/ fails and shows error alert</t>
-        </is>
-      </c>
-      <c r="H25" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>The valid Vietnamese number 0912345678 was rejected with “Số điện thoại không hợp lệ. Vui lòng nhập đúng 9-10 chữ số.”.</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -1906,10 +1938,14 @@
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
-        </is>
-      </c>
-      <c r="L25" s="2" t="inlineStr"/>
+          <t>Executed twice on Google Chrome 151 / Windows. The regex disallows the required leading zero.</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>bugs/evidence_images/bug_012_valid_phone_rejected.png</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1944,12 +1980,12 @@
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Profile updated successfully</t>
-        </is>
-      </c>
-      <c r="H26" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>The address was saved through the profile form; confirmation message: “Cập nhật thành công!”.</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -1964,7 +2000,7 @@
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
+          <t>Executed twice on Google Chrome 151 / Windows.</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr"/>
@@ -2002,17 +2038,17 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>Expands details with product list</t>
-        </is>
-      </c>
-      <c r="H27" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>Order-history rows provide no expansion control, details link, or item-level view.</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>BUG-016</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
@@ -2022,10 +2058,14 @@
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
-        </is>
-      </c>
-      <c r="L27" s="2" t="inlineStr"/>
+          <t>Executed twice on Google Chrome 151 / Windows. The interface exposes only summary columns.</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>bugs/evidence_images/bug_016_order_history_has_no_details.png</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2060,12 +2100,12 @@
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Displays empty history message</t>
-        </is>
-      </c>
-      <c r="H28" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>The order-history empty state was displayed for a user with no orders at the start of execution.</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -2080,7 +2120,7 @@
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
+          <t>Executed twice on Google Chrome 151 / Windows.</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr"/>
@@ -2118,7 +2158,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>Renders order cards correctly</t>
+          <t>Not executed on a qualifying mobile environment.</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
@@ -2138,7 +2178,7 @@
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
+          <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr"/>
@@ -2176,7 +2216,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Web shows 'Hủy đơn' during shipping while Mobile hides it</t>
+          <t>Not executed on a qualifying mobile environment.</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
@@ -2196,7 +2236,7 @@
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
+          <t>The Web behavior was inspected, but the comparison requires execution of the Mobile app.</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr"/>
@@ -2234,12 +2274,12 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Renders summary metric cards</t>
-        </is>
-      </c>
-      <c r="H31" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>Dashboard displayed revenue and order-count summary cards.</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
@@ -2254,7 +2294,7 @@
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
+          <t>Executed twice on Google Chrome 151 / Windows.</t>
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr"/>
@@ -2292,17 +2332,17 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Revenue metric multiplies delivered total by 2 (o.total_amount * 2), doubling total revenue</t>
-        </is>
-      </c>
-      <c r="H32" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>Delivered-order revenue should total 8,234,567 ₫; the dashboard rendered Tổng doanh thu (Delivered) 16.469.134 ₫.</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>BUG-013</t>
+          <t>BUG-014</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
@@ -2312,10 +2352,14 @@
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
-        </is>
-      </c>
-      <c r="L32" s="2" t="inlineStr"/>
+          <t>Executed twice on Google Chrome 151 / Windows. The reducer multiplies each delivered total by two.</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>bugs/evidence_images/bug_014_admin_revenue_doubled.png</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2350,12 +2394,12 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Renders cell via dangerouslySetInnerHTML={{ __html: o.shipping_address }}, executing arbitrary script</t>
-        </is>
-      </c>
-      <c r="H33" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>Stored shipping-address HTML was interpreted as markup in the Admin Orders table.</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
@@ -2370,10 +2414,14 @@
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
-        </is>
-      </c>
-      <c r="L33" s="2" t="inlineStr"/>
+          <t>Executed twice on Google Chrome 151 / Windows. dangerouslySetInnerHTML permits stored script-capable content.</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>bugs/evidence_images/bug_013_stored_html_injection.png</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2408,12 +2456,12 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Status update buttons displayed per order row</t>
-        </is>
-      </c>
-      <c r="H34" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>The pending order exposed the expected actions: Xác nhận, Hủy.</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
@@ -2428,7 +2476,7 @@
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
+          <t>Executed twice on Google Chrome 151 / Windows.</t>
         </is>
       </c>
       <c r="L34" s="2" t="inlineStr"/>
@@ -2466,12 +2514,12 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Sidebar tabs switch content smoothly</t>
-        </is>
-      </c>
-      <c r="H35" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>All six primary admin navigation destinations were visible and selectable.</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
@@ -2486,7 +2534,7 @@
       </c>
       <c r="K35" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
+          <t>Executed twice on Google Chrome 151 / Windows.</t>
         </is>
       </c>
       <c r="L35" s="2" t="inlineStr"/>
@@ -2524,17 +2572,17 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Toast notification displayed</t>
-        </is>
-      </c>
-      <c r="H36" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>The status changed to Đã xác nhận, but no success toast or confirmation message appeared.</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>BUG-019</t>
         </is>
       </c>
       <c r="J36" s="2" t="inlineStr">
@@ -2544,10 +2592,14 @@
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
-        </is>
-      </c>
-      <c r="L36" s="2" t="inlineStr"/>
+          <t>Executed twice on Google Chrome 151 / Windows. State change feedback is limited to the table badge update.</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>bugs/evidence_images/bug_019_admin_status_no_success_feedback.png</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2582,17 +2634,17 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Code sets fakeMassUpdatedProducts, overwriting all product names with edited name</t>
-        </is>
-      </c>
-      <c r="H37" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>Editing one product changed every visible product name in client state.</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>BUG-017</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
@@ -2602,10 +2654,14 @@
       </c>
       <c r="K37" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
-        </is>
-      </c>
-      <c r="L37" s="2" t="inlineStr"/>
+          <t>Executed twice on Google Chrome 151 / Windows. The success handler maps the edited name onto every product.</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>bugs/evidence_images/bug_017_admin_product_edit_corrupts_list.png</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2640,17 +2696,17 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Displays loading indicator while fetching</t>
-        </is>
-      </c>
-      <c r="H38" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>No loading spinner, progress indicator, or loading message appeared while Admin APIs were deliberately delayed.</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>Failed</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>BUG-018</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
@@ -2660,10 +2716,14 @@
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
-        </is>
-      </c>
-      <c r="L38" s="2" t="inlineStr"/>
+          <t>Executed twice on Google Chrome 151 / Windows. The interface renders empty/default content during data retrieval.</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>bugs/evidence_images/bug_018_admin_missing_loading_indicator.png</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2673,7 +2733,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>FR-23</t>
+          <t>Pool D</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -2698,7 +2758,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Image uses resizeMode='stretch', distorting non-square product images</t>
+          <t>Not executed on a qualifying mobile environment.</t>
         </is>
       </c>
       <c r="H39" s="3" t="inlineStr">
@@ -2718,7 +2778,7 @@
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
+          <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr"/>
@@ -2731,7 +2791,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>FR-23</t>
+          <t>Pool D</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -2756,7 +2816,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Category name omitted entirely despite category_id present in API response</t>
+          <t>Not executed on a qualifying mobile environment.</t>
         </is>
       </c>
       <c r="H40" s="3" t="inlineStr">
@@ -2766,7 +2826,7 @@
       </c>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>BUG-004</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
@@ -2776,7 +2836,7 @@
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
+          <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr"/>
@@ -2789,7 +2849,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>FR-23</t>
+          <t>Pool D</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -2814,7 +2874,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Input field accepts numeric values</t>
+          <t>Not executed on a qualifying mobile environment.</t>
         </is>
       </c>
       <c r="H41" s="3" t="inlineStr">
@@ -2834,7 +2894,7 @@
       </c>
       <c r="K41" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
+          <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
         </is>
       </c>
       <c r="L41" s="2" t="inlineStr"/>
@@ -2847,7 +2907,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>FR-23</t>
+          <t>Pool D</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -2872,7 +2932,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Quantity defaults to 1 safely</t>
+          <t>Not executed on a qualifying mobile environment.</t>
         </is>
       </c>
       <c r="H42" s="3" t="inlineStr">
@@ -2892,7 +2952,7 @@
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
+          <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
         </is>
       </c>
       <c r="L42" s="2" t="inlineStr"/>
@@ -2905,7 +2965,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>FR-23</t>
+          <t>Pool D</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -2930,7 +2990,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Back button returns user to previous screen</t>
+          <t>Not executed on a qualifying mobile environment.</t>
         </is>
       </c>
       <c r="H43" s="3" t="inlineStr">
@@ -2950,7 +3010,7 @@
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
+          <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
         </is>
       </c>
       <c r="L43" s="2" t="inlineStr"/>
@@ -2963,7 +3023,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>FR-23</t>
+          <t>Pool D</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -2988,7 +3048,7 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Button text updates to 'Đã thêm' temporarily</t>
+          <t>Not executed on a qualifying mobile environment.</t>
         </is>
       </c>
       <c r="H44" s="3" t="inlineStr">
@@ -3008,7 +3068,7 @@
       </c>
       <c r="K44" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
+          <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
         </is>
       </c>
       <c r="L44" s="2" t="inlineStr"/>
@@ -3021,7 +3081,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>FR-23</t>
+          <t>Pool D</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -3046,7 +3106,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Displays technical error 'Sản phẩm không tồn tại (Lỗi trắng trang do data rỗng)' without navigation CTA</t>
+          <t>Not executed on a qualifying mobile environment.</t>
         </is>
       </c>
       <c r="H45" s="3" t="inlineStr">
@@ -3056,7 +3116,7 @@
       </c>
       <c r="I45" s="2" t="inlineStr">
         <is>
-          <t>BUG-005</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
@@ -3066,7 +3126,7 @@
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
+          <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
         </is>
       </c>
       <c r="L45" s="2" t="inlineStr"/>
@@ -3079,7 +3139,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>FR-23</t>
+          <t>Pool D</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -3104,7 +3164,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Price formatted cleanly on screen</t>
+          <t>Not executed on a qualifying mobile environment.</t>
         </is>
       </c>
       <c r="H46" s="3" t="inlineStr">
@@ -3124,7 +3184,7 @@
       </c>
       <c r="K46" s="2" t="inlineStr">
         <is>
-          <t>Requires verification against the running SUT.</t>
+          <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
         </is>
       </c>
       <c r="L46" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
test(hw03): enforce complete checklist schema
</commit_message>
<xml_diff>
--- a/docs/assignments/HW03/deliverables/checklist/gui_checklist.xlsx
+++ b/docs/assignments/HW03/deliverables/checklist/gui_checklist.xlsx
@@ -10,9 +10,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GUI Checklist" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'GUI Checklist'!$A$1:$L$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'GUI Checklist'!$A$1:$O$46</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'GUI Checklist'!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'GUI Checklist'!$A$1:$L$46</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'GUI Checklist'!$A$1:$O$46</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -440,21 +440,24 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L46"/>
+  <dimension ref="A1:O46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="11" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
     <col width="42" customWidth="1" min="5" max="5"/>
     <col width="42" customWidth="1" min="6" max="6"/>
     <col width="42" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
     <col width="42" customWidth="1" min="10" max="10"/>
-    <col width="42" customWidth="1" min="11" max="11"/>
-    <col width="42" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="42" customWidth="1" min="13" max="13"/>
+    <col width="42" customWidth="1" min="14" max="14"/>
+    <col width="42" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -475,45 +478,60 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Screen</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>Test Item Description</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Preconditions</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Bug ID</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Origin</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>AI Critique / Reason Missed</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Evidence Reference</t>
         </is>
@@ -537,45 +555,60 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>Web Cart</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
           <t>Check Web Cart table columns alignment, currency formatting (X,XXX ₫), and total summary display</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Cart contains items</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Table displays Product, Price, Quantity, Subtotal, Actions with currency formatted in ₫</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="2" t="inlineStr">
         <is>
           <t>Cart rendered 5 columns (Sản phẩm, Giá, Số lượng, Thành tiền, Thao tác) and displayed the formatted total.</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Google Chrome 151 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr">
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
         <is>
           <t>Standard static UI layout correctly recognized by AI model during visual DOM inspection.</t>
         </is>
       </c>
-      <c r="K2" s="2" t="inlineStr">
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>Executed twice on Google Chrome 151 / Windows.</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr"/>
+      <c r="O2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -595,45 +628,60 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
+          <t>Web Product Detail</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
           <t>Verify Web ProductDetail 'Thêm vào giỏ hàng' button action on first click</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Product detail page loaded</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>First click on 'Thêm vào giỏ hàng' adds 1 item to cart state immediately</t>
         </is>
       </c>
-      <c r="G3" s="2" t="inlineStr">
+      <c r="H3" s="2" t="inlineStr">
         <is>
           <t>After one click on Product Detail, the cart remained empty; a second click is required.</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
+      <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Google Chrome 151 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
         <is>
           <t>BUG-001</t>
         </is>
       </c>
-      <c r="J3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>AI missed this because static DOM analysis showed an onClick handler bound to the button; AI assumed single-click handlers always dispatch state updates without checking state machine internal event counters.</t>
         </is>
       </c>
-      <c r="K3" s="2" t="inlineStr">
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>Executed twice on Google Chrome 151 / Windows. First click does not add the product.</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="O3" s="2" t="inlineStr">
         <is>
           <t>bugs/evidence_images/bug_001_first_click_cart_empty.png</t>
         </is>
@@ -657,45 +705,60 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
+          <t>Web Cart</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
           <t>Validate cart input rejection of zero and negative quantities (0, -5)</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>User in Cart view</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>Inputting 0 or negative numbers shows validation error or defaults to 1</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="H4" s="2" t="inlineStr">
         <is>
           <t>The product was added with quantity -5 and a negative subtotal (iPhone 15 Pro Max 30.000.000 ₫ -5 -150.000.000 ₫ Xóa).</t>
         </is>
       </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Google Chrome 151 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
         <is>
           <t>BUG-002</t>
         </is>
       </c>
-      <c r="J4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>AI missed boundary value validation on numeric inputs because standard HTML5 number inputs without min attribute are assumed valid by LLMs unless explicitly tested with negative boundary values.</t>
         </is>
       </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>Executed twice on Google Chrome 151 / Windows. No minimum or validation feedback is provided.</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="O4" s="2" t="inlineStr">
         <is>
           <t>bugs/evidence_images/bug_002_negative_quantity.png</t>
         </is>
@@ -719,45 +782,60 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
+          <t>Web Cart</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
           <t>Validate cart handling of decimal quantity input (e.g. 2.5)</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>User in Cart view</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>Entering decimal values displays error notification 'Số lượng phải là số nguyên'</t>
         </is>
       </c>
-      <c r="G5" s="2" t="inlineStr">
+      <c r="H5" s="2" t="inlineStr">
         <is>
           <t>Entering 2.5 produced cart quantity 2 without any validation message.</t>
         </is>
       </c>
-      <c r="H5" s="2" t="inlineStr">
+      <c r="I5" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Google Chrome 151 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
         <is>
           <t>BUG-003</t>
         </is>
       </c>
-      <c r="J5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>AI missed silent truncation because parseInt() converts 2.5 to 2 without throwing a runtime error, masking the invalid input behavior during basic path testing.</t>
         </is>
       </c>
-      <c r="K5" s="2" t="inlineStr">
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>Executed twice on Google Chrome 151 / Windows. The decimal was silently truncated by parseInt().</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="O5" s="2" t="inlineStr">
         <is>
           <t>bugs/evidence_images/bug_003_decimal_quantity_truncated.png</t>
         </is>
@@ -781,45 +859,60 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
+          <t>Web Checkout</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
           <t>Verify Web Checkout total amount input field read-only status</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Cart containing items, navigating to /checkout</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Total amount display field is read-only or non-editable text</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="H6" s="2" t="inlineStr">
         <is>
           <t>Checkout total is rendered in an editable number input and accepted manual changes.</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="I6" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Google Chrome 151 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
         <is>
           <t>BUG-006</t>
         </is>
       </c>
-      <c r="J6" s="2" t="inlineStr">
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>AI missed this security flaw because total summary boxes are visually styled like read-only fields; code review without input element attribute checks failed to spot type='number' without readOnly.</t>
         </is>
       </c>
-      <c r="K6" s="2" t="inlineStr">
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>Executed twice on Google Chrome 151 / Windows. The displayed/payment total is client-editable.</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="O6" s="2" t="inlineStr">
         <is>
           <t>bugs/evidence_images/bug_006_editable_checkout_total.png</t>
         </is>
@@ -843,45 +936,60 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
+          <t>Web Cart</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
           <t>Verify Web Cart '← Mua tiếp' and 'Tiến hành thanh toán' navigation links</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>User in Cart view with items</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>'← Mua tiếp' redirects to /; 'Tiến hành thanh toán' opens /checkout</t>
         </is>
       </c>
-      <c r="G7" s="2" t="inlineStr">
+      <c r="H7" s="2" t="inlineStr">
         <is>
           <t>Continue shopping links to the product list and the checkout control is available.</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
+      <c r="I7" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Google Chrome 151 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J7" s="2" t="inlineStr">
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>Standard React Router &lt;Link&gt; and navigate() routes parsed accurately by AI.</t>
         </is>
       </c>
-      <c r="K7" s="2" t="inlineStr">
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>Executed twice on Google Chrome 151 / Windows.</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr"/>
+      <c r="O7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -901,45 +1009,60 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
+          <t>Web Checkout</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
           <t>Verify Web Checkout unauthenticated user access redirection</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Unauthenticated user clicks Checkout</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Triggers login modal/alert and redirects to /login</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="H8" s="2" t="inlineStr">
         <is>
           <t>Unauthenticated checkout displayed “Bạn cần đăng nhập để thanh toán!” and redirected to /login.</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="I8" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Google Chrome 151 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J8" s="2" t="inlineStr">
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>Authentication check logic correctly mapped from auth context.</t>
         </is>
       </c>
-      <c r="K8" s="2" t="inlineStr">
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>Executed twice on Google Chrome 151 / Windows.</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr"/>
+      <c r="O8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -959,45 +1082,60 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
+          <t>Web Cart</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
           <t>Verify Web Cart empty state display when cart is cleared</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Cart emptied</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>Displays 'Giỏ hàng của bạn đang trống' with CTA button 'Tiếp tục mua sắm'</t>
         </is>
       </c>
-      <c r="G9" s="2" t="inlineStr">
+      <c r="H9" s="2" t="inlineStr">
         <is>
           <t>The empty-cart message and continue-shopping link were displayed after removing the item.</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
+      <c r="I9" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Google Chrome 151 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J9" s="2" t="inlineStr">
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>Empty state conditionally rendered when cart.length === 0.</t>
         </is>
       </c>
-      <c r="K9" s="2" t="inlineStr">
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>Executed twice on Google Chrome 151 / Windows.</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr"/>
+      <c r="O9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1017,45 +1155,60 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
+          <t>Web Cart / Checkout</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
           <t>Verify cart clearing in Web CartContext after successful checkout payment</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>User completes order payment on Web Checkout</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Cart is cleared from React state and localStorage; header badge updates to 0</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="H10" s="2" t="inlineStr">
         <is>
           <t>The purchased item remained in the cart after checkout completed.</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="I10" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Google Chrome 151 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
         <is>
           <t>BUG-007</t>
         </is>
       </c>
-      <c r="J10" s="2" t="inlineStr">
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>AI missed missing state reset call because checkout success handler executed navigation redirect without verifying context state disposal (clearCart()).</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>Executed twice on Google Chrome 151 / Windows. Checkout does not invoke clearCart().</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="O10" s="2" t="inlineStr">
         <is>
           <t>bugs/evidence_images/bug_007_cart_retained_after_checkout.png</t>
         </is>
@@ -1079,45 +1232,60 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
+          <t>Mobile Cart</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
           <t>Check Mobile Cart layout item row formatting and total sum calculation</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Mobile app cart screen</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>ScrollView lists cart items with unit price, quantity edit, item total, and remove button</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
+      <c r="H11" s="2" t="inlineStr">
         <is>
           <t>Not executed on a qualifying mobile environment.</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Qualifying real mobile device or approved cloud device — pending execution</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J11" s="2" t="inlineStr">
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>Mobile React Native component hierarchy correctly analyzed.</t>
         </is>
       </c>
-      <c r="K11" s="2" t="inlineStr">
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr"/>
+      <c r="O11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1137,45 +1305,60 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
+          <t>Mobile Cart</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
           <t>Verify Mobile Cart quantity input change behavior when typing a new number</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Mobile cart screen</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>Typing quantity N sets item quantity to N</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>Not executed on a qualifying mobile environment.</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
+      <c r="I12" s="3" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Qualifying real mobile device or approved cloud device — pending execution</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>AI missed off-by-one arithmetic bug in input change handler because parsed + 1 was misconstrued as an increment button handler rather than direct text input parsing.</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr"/>
+      <c r="O12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1195,45 +1378,60 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
+          <t>Mobile Checkout</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
           <t>Verify Mobile Checkout payload creation with multi-item cart</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Mobile cart with &gt;1 items</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>Full cart array sent in API POST request body</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Not executed on a qualifying mobile environment.</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="I13" s="3" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Qualifying real mobile device or approved cloud device — pending execution</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J13" s="2" t="inlineStr">
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>AI missed payload array truncation because slice(0, -1) is syntactically clean JavaScript; AI assumed array slicing was used for defensive copying rather than unintended item removal.</t>
         </is>
       </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr"/>
+      <c r="O13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1253,45 +1451,60 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
+          <t>Mobile Cart</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
           <t>Check Mobile Cart remove item swipe/button confirmation feedback</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Mobile cart item row</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>Clicking 'Xóa' removes item immediately and updates cart badge</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="H14" s="2" t="inlineStr">
         <is>
           <t>Not executed on a qualifying mobile environment.</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
+      <c r="I14" s="3" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Qualifying real mobile device or approved cloud device — pending execution</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J14" s="2" t="inlineStr">
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
         <is>
           <t>Mobile array filter state update verified.</t>
         </is>
       </c>
-      <c r="K14" s="2" t="inlineStr">
+      <c r="N14" s="2" t="inlineStr">
         <is>
           <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr"/>
+      <c r="O14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1311,45 +1524,60 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
+          <t>Order Lifecycle</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
           <t>Check initial order status badge rendering upon successful order placement</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>Order created</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>Status badge displays 'Chờ xác nhận' (pending) with yellow status highlight</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
+      <c r="H15" s="2" t="inlineStr">
         <is>
           <t>A newly created order displayed “Chờ xác nhận” with the pending badge style.</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="I15" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Google Chrome 151 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J15" s="2" t="inlineStr">
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
         <is>
           <t>Default initial state pending verified.</t>
         </is>
       </c>
-      <c r="K15" s="2" t="inlineStr">
+      <c r="N15" s="2" t="inlineStr">
         <is>
           <t>Executed twice on Google Chrome 151 / Windows.</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr"/>
+      <c r="O15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1369,45 +1597,60 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
+          <t>Order Lifecycle</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
           <t>Verify valid state transition sequence: pending -&gt; confirmed -&gt; shipping -&gt; delivered</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>Admin user logged in</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>Transitions execute sequentially; status updates on UI with appropriate colors</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>The API accepted the valid sequence confirmed → shipping → delivered.</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="I16" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Google Chrome 151 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J16" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>Happy path state machine transitions operating as designed.</t>
         </is>
       </c>
-      <c r="K16" s="2" t="inlineStr">
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>Executed twice on Google Chrome 151 / Windows.</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr"/>
+      <c r="O16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1427,45 +1670,60 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
+          <t>Order Lifecycle</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
           <t>Validate user order cancellation rule for orders in shipping state</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>User order with status shipping</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>Cancellation is rejected with error 'Không thể hủy đơn hàng đang giao'</t>
         </is>
       </c>
-      <c r="G17" s="2" t="inlineStr">
+      <c r="H17" s="2" t="inlineStr">
         <is>
           <t>The cancellation request returned HTTP 200; the shipping order became canceled.</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
+      <c r="I17" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Google Chrome 151 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
         <is>
           <t>BUG-010</t>
         </is>
       </c>
-      <c r="J17" s="2" t="inlineStr">
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>AI missed state machine boundary violation because backend logic checked status === 'delivered' || status === 'canceled' using negative logic instead of positive whitelist (status === 'pending' || status === 'confirmed').</t>
         </is>
       </c>
-      <c r="K17" s="2" t="inlineStr">
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>Executed twice on Google Chrome 151 / Windows. Shipping is incorrectly treated as cancelable.</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr">
+      <c r="O17" s="2" t="inlineStr">
         <is>
           <t>bugs/evidence_images/bug_010_shipping_order_canceled.png</t>
         </is>
@@ -1489,45 +1747,60 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
+          <t>Order Lifecycle</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
           <t>Validate admin state machine restriction on transitioning canceled orders to delivered</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Order status is canceled</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>Admin UI disables transition and API rejects request with HTTP 400</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="H18" s="2" t="inlineStr">
         <is>
           <t>Canceled → delivered returned HTTP 200; the admin UI displayed the resulting delivered state.</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="I18" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Google Chrome 151 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
         <is>
           <t>BUG-011</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>AI missed illegal terminal state escape because API code explicitly added if (currentStatus === 'canceled' &amp;&amp; status === 'delivered') isValidTransition = true, violating business logic.</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>Executed twice on Google Chrome 151 / Windows. A terminal canceled order can escape to delivered.</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="O18" s="2" t="inlineStr">
         <is>
           <t>bugs/evidence_images/bug_011_canceled_order_delivered.png</t>
         </is>
@@ -1551,45 +1824,60 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
+          <t>Web Checkout</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
           <t>Validate Coupon code application form on Checkout</t>
         </is>
       </c>
-      <c r="E19" s="2" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>Valid discount coupon entered</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>Total amount updates with discount value and success toast is displayed</t>
         </is>
       </c>
-      <c r="G19" s="2" t="inlineStr">
+      <c r="H19" s="2" t="inlineStr">
         <is>
           <t>SAVE10 (10%) reported savings of -270,000,000 ₫ and a final total of 300,000,000 ₫; the correct values are 3,000,000 ₫ and 27,000,000 ₫.</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
+      <c r="I19" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>Google Chrome 151 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
         <is>
           <t>BUG-015</t>
         </is>
       </c>
-      <c r="J19" s="2" t="inlineStr">
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
         <is>
           <t>Form submit handler and coupon calculation verified.</t>
         </is>
       </c>
-      <c r="K19" s="2" t="inlineStr">
+      <c r="N19" s="2" t="inlineStr">
         <is>
           <t>Executed twice on Google Chrome 151 / Windows. Percentage discount calculation is incorrect.</t>
         </is>
       </c>
-      <c r="L19" s="2" t="inlineStr">
+      <c r="O19" s="2" t="inlineStr">
         <is>
           <t>bugs/evidence_images/bug_015_percent_coupon_calculation.png</t>
         </is>
@@ -1613,45 +1901,60 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
+          <t>Web Checkout</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
           <t>Validate invalid coupon code feedback on Checkout</t>
         </is>
       </c>
-      <c r="E20" s="2" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Expired or non-existent coupon entered</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>Displays red error text 'Mã giảm giá không hợp lệ hoặc đã hết hạn'</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="H20" s="2" t="inlineStr">
         <is>
           <t>The invalid coupon displayed the inline message “Mã giảm giá không tồn tại hoặc đã bị vô hiệu hóa”.</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>Google Chrome 151 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J20" s="2" t="inlineStr">
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
         <is>
           <t>Error response handling verified.</t>
         </is>
       </c>
-      <c r="K20" s="2" t="inlineStr">
+      <c r="N20" s="2" t="inlineStr">
         <is>
           <t>Executed twice on Google Chrome 151 / Windows.</t>
         </is>
       </c>
-      <c r="L20" s="2" t="inlineStr"/>
+      <c r="O20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1671,45 +1974,60 @@
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
+          <t>Web Checkout</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
           <t>Check order confirmation screen navigation after successful order placement</t>
         </is>
       </c>
-      <c r="E21" s="2" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>Order form submitted</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>Redirects to /profile or Order Details with order summary</t>
         </is>
       </c>
-      <c r="G21" s="2" t="inlineStr">
+      <c r="H21" s="2" t="inlineStr">
         <is>
           <t>Checkout displayed a dedicated success state and provided navigation back to the home page.</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
+      <c r="I21" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>Google Chrome 151 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J21" s="2" t="inlineStr">
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
         <is>
           <t>Router redirect verified.</t>
         </is>
       </c>
-      <c r="K21" s="2" t="inlineStr">
+      <c r="N21" s="2" t="inlineStr">
         <is>
           <t>Executed twice on Google Chrome 151 / Windows.</t>
         </is>
       </c>
-      <c r="L21" s="2" t="inlineStr"/>
+      <c r="O21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1729,45 +2047,60 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
+          <t>Order Lifecycle</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
           <t>Check terminal state immutability for delivered orders</t>
         </is>
       </c>
-      <c r="E22" s="2" t="inlineStr">
+      <c r="F22" s="2" t="inlineStr">
         <is>
           <t>Order status delivered</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>Action buttons (Cancel, Update Status) are disabled/hidden</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="H22" s="2" t="inlineStr">
         <is>
           <t>A delivered order rejected a transition back to confirmed with HTTP 400.</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="I22" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="I22" s="2" t="inlineStr">
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>Google Chrome 151 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J22" s="2" t="inlineStr">
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
         <is>
           <t>Terminal state handling for delivered orders verified.</t>
         </is>
       </c>
-      <c r="K22" s="2" t="inlineStr">
+      <c r="N22" s="2" t="inlineStr">
         <is>
           <t>Executed twice on Google Chrome 151 / Windows.</t>
         </is>
       </c>
-      <c r="L22" s="2" t="inlineStr"/>
+      <c r="O22" s="2" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1787,45 +2120,60 @@
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
+          <t>Web Order History</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
           <t>Check Web Profile Order History table responsiveness and layout</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="F23" s="2" t="inlineStr">
         <is>
           <t>Web Profile page open</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>Two-column desktop layout (Profile info on left, Order history on right)</t>
         </is>
       </c>
-      <c r="G23" s="2" t="inlineStr">
+      <c r="H23" s="2" t="inlineStr">
         <is>
           <t>Order history rendered as a structured five-column table at 1440×1000.</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr">
+      <c r="I23" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="I23" s="2" t="inlineStr">
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Google Chrome 151 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J23" s="2" t="inlineStr">
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
         <is>
           <t>Tailwind CSS flex/grid layout verified.</t>
         </is>
       </c>
-      <c r="K23" s="2" t="inlineStr">
+      <c r="N23" s="2" t="inlineStr">
         <is>
           <t>Executed twice on Google Chrome 151 / Windows.</t>
         </is>
       </c>
-      <c r="L23" s="2" t="inlineStr"/>
+      <c r="O23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1845,45 +2193,60 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
+          <t>Web Order History</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
           <t>Verify status badge color mapping in Order History table</t>
         </is>
       </c>
-      <c r="E24" s="2" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
         <is>
           <t>Orders with various statuses</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>pending: yellow, confirmed: indigo, shipping: blue, delivered: green, canceled: red</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="H24" s="2" t="inlineStr">
         <is>
           <t>Status badges rendered localized labels: Đã hủy, Đã giao, Chờ xác nhận, Chờ xác nhận.</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr">
+      <c r="I24" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="I24" s="2" t="inlineStr">
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>Google Chrome 151 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J24" s="2" t="inlineStr">
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
         <is>
           <t>Status color mapping dictionary verified.</t>
         </is>
       </c>
-      <c r="K24" s="2" t="inlineStr">
+      <c r="N24" s="2" t="inlineStr">
         <is>
           <t>Executed twice on Google Chrome 151 / Windows.</t>
         </is>
       </c>
-      <c r="L24" s="2" t="inlineStr"/>
+      <c r="O24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1903,45 +2266,60 @@
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
+          <t>Web User Profile</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
           <t>Validate User Profile phone number validation with standard Vietnamese phone number (e.g. 0912345678)</t>
         </is>
       </c>
-      <c r="E25" s="2" t="inlineStr">
+      <c r="F25" s="2" t="inlineStr">
         <is>
           <t>User editing profile phone field</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
+      <c r="G25" s="2" t="inlineStr">
         <is>
           <t>Phone starting with 0 accepted and saved successfully</t>
         </is>
       </c>
-      <c r="G25" s="2" t="inlineStr">
+      <c r="H25" s="2" t="inlineStr">
         <is>
           <t>The valid Vietnamese number 0912345678 was rejected with “Số điện thoại không hợp lệ. Vui lòng nhập đúng 9-10 chữ số.”.</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr">
+      <c r="I25" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
-      <c r="I25" s="2" t="inlineStr">
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>Google Chrome 151 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
         <is>
           <t>BUG-012</t>
         </is>
       </c>
-      <c r="J25" s="2" t="inlineStr">
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
         <is>
           <t>AI missed regex logic flaw because [1-9] pattern looked like a valid numeric range constraint, ignoring Vietnamese phone numbering standard where 100% of mobile numbers start with 0.</t>
         </is>
       </c>
-      <c r="K25" s="2" t="inlineStr">
+      <c r="N25" s="2" t="inlineStr">
         <is>
           <t>Executed twice on Google Chrome 151 / Windows. The regex disallows the required leading zero.</t>
         </is>
       </c>
-      <c r="L25" s="2" t="inlineStr">
+      <c r="O25" s="2" t="inlineStr">
         <is>
           <t>bugs/evidence_images/bug_012_valid_phone_rejected.png</t>
         </is>
@@ -1965,45 +2343,60 @@
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
+          <t>Web User Profile</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
           <t>Validate User Profile address update input field text saving</t>
         </is>
       </c>
-      <c r="E26" s="2" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
         <is>
           <t>User entering new shipping address</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>Input accepted and saved via PUT /api/user/profile</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="H26" s="2" t="inlineStr">
         <is>
           <t>The address was saved through the profile form; confirmation message: “Cập nhật thành công!”.</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="I26" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr">
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Google Chrome 151 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J26" s="2" t="inlineStr">
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
         <is>
           <t>Form state binding verified.</t>
         </is>
       </c>
-      <c r="K26" s="2" t="inlineStr">
+      <c r="N26" s="2" t="inlineStr">
         <is>
           <t>Executed twice on Google Chrome 151 / Windows.</t>
         </is>
       </c>
-      <c r="L26" s="2" t="inlineStr"/>
+      <c r="O26" s="2" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2023,45 +2416,60 @@
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
+          <t>Web Order History</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
           <t>Check Order History list item click expansion / details view</t>
         </is>
       </c>
-      <c r="E27" s="2" t="inlineStr">
+      <c r="F27" s="2" t="inlineStr">
         <is>
           <t>Order item clicked</t>
         </is>
       </c>
-      <c r="F27" s="2" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>Expands row or opens order details modal with item breakdown</t>
         </is>
       </c>
-      <c r="G27" s="2" t="inlineStr">
+      <c r="H27" s="2" t="inlineStr">
         <is>
           <t>Order-history rows provide no expansion control, details link, or item-level view.</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr">
+      <c r="I27" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr">
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>Google Chrome 151 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
         <is>
           <t>BUG-016</t>
         </is>
       </c>
-      <c r="J27" s="2" t="inlineStr">
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
         <is>
           <t>Navigation / toggle state verified.</t>
         </is>
       </c>
-      <c r="K27" s="2" t="inlineStr">
+      <c r="N27" s="2" t="inlineStr">
         <is>
           <t>Executed twice on Google Chrome 151 / Windows. The interface exposes only summary columns.</t>
         </is>
       </c>
-      <c r="L27" s="2" t="inlineStr">
+      <c r="O27" s="2" t="inlineStr">
         <is>
           <t>bugs/evidence_images/bug_016_order_history_has_no_details.png</t>
         </is>
@@ -2085,45 +2493,60 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
+          <t>Web Order History</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
           <t>Verify empty state rendering when user has 0 orders</t>
         </is>
       </c>
-      <c r="E28" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
         <is>
           <t>New account with no orders</t>
         </is>
       </c>
-      <c r="F28" s="2" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>Displays 'Bạn chưa có đơn hàng nào.'</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="H28" s="2" t="inlineStr">
         <is>
           <t>The order-history empty state was displayed for a user with no orders at the start of execution.</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="I28" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="I28" s="2" t="inlineStr">
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>Google Chrome 151 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J28" s="2" t="inlineStr">
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
         <is>
           <t>Empty state condition orders.length === 0 verified.</t>
         </is>
       </c>
-      <c r="K28" s="2" t="inlineStr">
+      <c r="N28" s="2" t="inlineStr">
         <is>
           <t>Executed twice on Google Chrome 151 / Windows.</t>
         </is>
       </c>
-      <c r="L28" s="2" t="inlineStr"/>
+      <c r="O28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2143,45 +2566,60 @@
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
+          <t>Mobile Profile</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
           <t>Check Mobile Profile order cards summary display</t>
         </is>
       </c>
-      <c r="E29" s="2" t="inlineStr">
+      <c r="F29" s="2" t="inlineStr">
         <is>
           <t>Mobile Profile screen</t>
         </is>
       </c>
-      <c r="F29" s="2" t="inlineStr">
+      <c r="G29" s="2" t="inlineStr">
         <is>
           <t>ScrollView displays order card with ID, Date, Formatted Amount, and Status</t>
         </is>
       </c>
-      <c r="G29" s="2" t="inlineStr">
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>Not executed on a qualifying mobile environment.</t>
         </is>
       </c>
-      <c r="H29" s="3" t="inlineStr">
+      <c r="I29" s="3" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="I29" s="2" t="inlineStr">
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>Qualifying real mobile device or approved cloud device — pending execution</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J29" s="2" t="inlineStr">
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
         <is>
           <t>Mobile React Native component verified.</t>
         </is>
       </c>
-      <c r="K29" s="2" t="inlineStr">
+      <c r="N29" s="2" t="inlineStr">
         <is>
           <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
         </is>
       </c>
-      <c r="L29" s="2" t="inlineStr"/>
+      <c r="O29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2201,45 +2639,60 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
+          <t>Mobile Profile</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
           <t>Check Web vs Mobile 'Hủy đơn' button visibility inconsistency</t>
         </is>
       </c>
-      <c r="E30" s="2" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
         <is>
           <t>Order in shipping state viewed on Mobile vs Web</t>
         </is>
       </c>
-      <c r="F30" s="2" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>Button visibility consistent across platforms (hidden for shipping)</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="H30" s="2" t="inlineStr">
         <is>
           <t>Not executed on a qualifying mobile environment.</t>
         </is>
       </c>
-      <c r="H30" s="3" t="inlineStr">
+      <c r="I30" s="3" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="I30" s="2" t="inlineStr">
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>Qualifying real mobile device or approved cloud device — pending execution</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J30" s="2" t="inlineStr">
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
         <is>
           <t>UI rendering discrepancy noted between web profile and mobile profile.</t>
         </is>
       </c>
-      <c r="K30" s="2" t="inlineStr">
+      <c r="N30" s="2" t="inlineStr">
         <is>
           <t>The Web behavior was inspected, but the comparison requires execution of the Mobile app.</t>
         </is>
       </c>
-      <c r="L30" s="2" t="inlineStr"/>
+      <c r="O30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2259,45 +2712,60 @@
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
+          <t>Admin Dashboard</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
           <t>Check Admin Dashboard layout summary metrics cards display</t>
         </is>
       </c>
-      <c r="E31" s="2" t="inlineStr">
+      <c r="F31" s="2" t="inlineStr">
         <is>
           <t>Admin Dashboard tab active</t>
         </is>
       </c>
-      <c r="F31" s="2" t="inlineStr">
+      <c r="G31" s="2" t="inlineStr">
         <is>
           <t>Renders metrics cards for Total Revenue, Total Orders, Total Products</t>
         </is>
       </c>
-      <c r="G31" s="2" t="inlineStr">
+      <c r="H31" s="2" t="inlineStr">
         <is>
           <t>Dashboard displayed revenue and order-count summary cards.</t>
         </is>
       </c>
-      <c r="H31" s="2" t="inlineStr">
+      <c r="I31" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="I31" s="2" t="inlineStr">
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>Google Chrome 151 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J31" s="2" t="inlineStr">
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
         <is>
           <t>Admin Dashboard grid structure verified.</t>
         </is>
       </c>
-      <c r="K31" s="2" t="inlineStr">
+      <c r="N31" s="2" t="inlineStr">
         <is>
           <t>Executed twice on Google Chrome 151 / Windows.</t>
         </is>
       </c>
-      <c r="L31" s="2" t="inlineStr"/>
+      <c r="O31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2317,45 +2785,60 @@
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
+          <t>Admin Dashboard</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
           <t>Verify Admin Dashboard Total Revenue calculation for delivered orders</t>
         </is>
       </c>
-      <c r="E32" s="2" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
         <is>
           <t>Delivered orders in system</t>
         </is>
       </c>
-      <c r="F32" s="2" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>Total Revenue equals sum of delivered orders total_amount</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="H32" s="2" t="inlineStr">
         <is>
           <t>Delivered-order revenue should total 8,234,567 ₫; the dashboard rendered Tổng doanh thu (Delivered) 16.469.134 ₫.</t>
         </is>
       </c>
-      <c r="H32" s="2" t="inlineStr">
+      <c r="I32" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
-      <c r="I32" s="2" t="inlineStr">
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>Google Chrome 151 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
         <is>
           <t>BUG-014</t>
         </is>
       </c>
-      <c r="J32" s="2" t="inlineStr">
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
         <is>
           <t>AI missed multiplication bug (* 2) in revenue accumulator callback because arithmetic expressions inside .reduce() require execution trace testing to spot arbitrary multiplier bugs.</t>
         </is>
       </c>
-      <c r="K32" s="2" t="inlineStr">
+      <c r="N32" s="2" t="inlineStr">
         <is>
           <t>Executed twice on Google Chrome 151 / Windows. The reducer multiplies each delivered total by two.</t>
         </is>
       </c>
-      <c r="L32" s="2" t="inlineStr">
+      <c r="O32" s="2" t="inlineStr">
         <is>
           <t>bugs/evidence_images/bug_014_admin_revenue_doubled.png</t>
         </is>
@@ -2379,45 +2862,60 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
+          <t>Admin Order Management</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
           <t>Verify Admin Order Management shipping address column HTML escaping (Stored XSS vulnerability test)</t>
         </is>
       </c>
-      <c r="E33" s="2" t="inlineStr">
+      <c r="F33" s="2" t="inlineStr">
         <is>
           <t>Order with shipping address containing &lt;img src=x onerror=alert(1)&gt;</t>
         </is>
       </c>
-      <c r="F33" s="2" t="inlineStr">
+      <c r="G33" s="2" t="inlineStr">
         <is>
           <t>HTML tags escaped; rendered as plain text in table cell</t>
         </is>
       </c>
-      <c r="G33" s="2" t="inlineStr">
+      <c r="H33" s="2" t="inlineStr">
         <is>
           <t>Stored shipping-address HTML was interpreted as markup in the Admin Orders table.</t>
         </is>
       </c>
-      <c r="H33" s="2" t="inlineStr">
+      <c r="I33" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
-      <c r="I33" s="2" t="inlineStr">
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>Google Chrome 151 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
         <is>
           <t>BUG-013</t>
         </is>
       </c>
-      <c r="J33" s="2" t="inlineStr">
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
         <is>
           <t>AI missed Stored XSS vulnerability because React code typically escapes JSX automatically; dangerouslySetInnerHTML usage without DOMPurify escaping requires explicit security audit rules.</t>
         </is>
       </c>
-      <c r="K33" s="2" t="inlineStr">
+      <c r="N33" s="2" t="inlineStr">
         <is>
           <t>Executed twice on Google Chrome 151 / Windows. dangerouslySetInnerHTML permits stored script-capable content.</t>
         </is>
       </c>
-      <c r="L33" s="2" t="inlineStr">
+      <c r="O33" s="2" t="inlineStr">
         <is>
           <t>bugs/evidence_images/bug_013_stored_html_injection.png</t>
         </is>
@@ -2441,45 +2939,60 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
+          <t>Admin Order Management</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
           <t>Check Admin Order Management status update dropdown/action buttons</t>
         </is>
       </c>
-      <c r="E34" s="2" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
         <is>
           <t>Admin viewing orders table</t>
         </is>
       </c>
-      <c r="F34" s="2" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>Buttons enabled for valid transitions only based on current status</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="H34" s="2" t="inlineStr">
         <is>
           <t>The pending order exposed the expected actions: Xác nhận, Hủy.</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr">
+      <c r="I34" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="I34" s="2" t="inlineStr">
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>Google Chrome 151 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J34" s="2" t="inlineStr">
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
         <is>
           <t>Table row action layout verified.</t>
         </is>
       </c>
-      <c r="K34" s="2" t="inlineStr">
+      <c r="N34" s="2" t="inlineStr">
         <is>
           <t>Executed twice on Google Chrome 151 / Windows.</t>
         </is>
       </c>
-      <c r="L34" s="2" t="inlineStr"/>
+      <c r="O34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2499,45 +3012,60 @@
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
+          <t>Admin Navigation</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
           <t>Check Admin Sidebar navigation menu items (Dashboard, Categories, Products, Coupons, Orders, Users)</t>
         </is>
       </c>
-      <c r="E35" s="2" t="inlineStr">
+      <c r="F35" s="2" t="inlineStr">
         <is>
           <t>Admin portal open</t>
         </is>
       </c>
-      <c r="F35" s="2" t="inlineStr">
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>Clicking menu items switches active view content without full page reload</t>
         </is>
       </c>
-      <c r="G35" s="2" t="inlineStr">
+      <c r="H35" s="2" t="inlineStr">
         <is>
           <t>All six primary admin navigation destinations were visible and selectable.</t>
         </is>
       </c>
-      <c r="H35" s="2" t="inlineStr">
+      <c r="I35" s="2" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
       </c>
-      <c r="I35" s="2" t="inlineStr">
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>Google Chrome 151 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J35" s="2" t="inlineStr">
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
         <is>
           <t>Sidebar routing verified.</t>
         </is>
       </c>
-      <c r="K35" s="2" t="inlineStr">
+      <c r="N35" s="2" t="inlineStr">
         <is>
           <t>Executed twice on Google Chrome 151 / Windows.</t>
         </is>
       </c>
-      <c r="L35" s="2" t="inlineStr"/>
+      <c r="O35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2557,45 +3085,60 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
+          <t>Admin Order Management</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
           <t>Verify status transition success toast message in Admin portal</t>
         </is>
       </c>
-      <c r="E36" s="2" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
         <is>
           <t>Admin updates order status</t>
         </is>
       </c>
-      <c r="F36" s="2" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>Toast notification 'Cập nhật trạng thái thành công' appears</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="H36" s="2" t="inlineStr">
         <is>
           <t>The status changed to Đã xác nhận, but no success toast or confirmation message appeared.</t>
         </is>
       </c>
-      <c r="H36" s="2" t="inlineStr">
+      <c r="I36" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
-      <c r="I36" s="2" t="inlineStr">
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>Google Chrome 151 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
         <is>
           <t>BUG-019</t>
         </is>
       </c>
-      <c r="J36" s="2" t="inlineStr">
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
         <is>
           <t>Notification feedback verified.</t>
         </is>
       </c>
-      <c r="K36" s="2" t="inlineStr">
+      <c r="N36" s="2" t="inlineStr">
         <is>
           <t>Executed twice on Google Chrome 151 / Windows. State change feedback is limited to the table badge update.</t>
         </is>
       </c>
-      <c r="L36" s="2" t="inlineStr">
+      <c r="O36" s="2" t="inlineStr">
         <is>
           <t>bugs/evidence_images/bug_019_admin_status_no_success_feedback.png</t>
         </is>
@@ -2619,45 +3162,60 @@
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
+          <t>Admin Product Management</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
           <t>Check Admin Product update state management when editing product name</t>
         </is>
       </c>
-      <c r="E37" s="2" t="inlineStr">
+      <c r="F37" s="2" t="inlineStr">
         <is>
           <t>Admin edits single product name in Admin form</t>
         </is>
       </c>
-      <c r="F37" s="2" t="inlineStr">
+      <c r="G37" s="2" t="inlineStr">
         <is>
           <t>Edits only target product in React state products array</t>
         </is>
       </c>
-      <c r="G37" s="2" t="inlineStr">
+      <c r="H37" s="2" t="inlineStr">
         <is>
           <t>Editing one product changed every visible product name in client state.</t>
         </is>
       </c>
-      <c r="H37" s="2" t="inlineStr">
+      <c r="I37" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
-      <c r="I37" s="2" t="inlineStr">
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>Google Chrome 151 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
         <is>
           <t>BUG-017</t>
         </is>
       </c>
-      <c r="J37" s="2" t="inlineStr">
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
         <is>
           <t>Product state mutation behavior verified.</t>
         </is>
       </c>
-      <c r="K37" s="2" t="inlineStr">
+      <c r="N37" s="2" t="inlineStr">
         <is>
           <t>Executed twice on Google Chrome 151 / Windows. The success handler maps the edited name onto every product.</t>
         </is>
       </c>
-      <c r="L37" s="2" t="inlineStr">
+      <c r="O37" s="2" t="inlineStr">
         <is>
           <t>bugs/evidence_images/bug_017_admin_product_edit_corrupts_list.png</t>
         </is>
@@ -2681,45 +3239,60 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
+          <t>Admin Order Management</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
           <t>Verify Admin Orders table loading spinner when fetching API data</t>
         </is>
       </c>
-      <c r="E38" s="2" t="inlineStr">
+      <c r="F38" s="2" t="inlineStr">
         <is>
           <t>Admin opens Orders tab</t>
         </is>
       </c>
-      <c r="F38" s="2" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>Displays 'Đang tải dữ liệu...' while HTTP GET is in progress</t>
         </is>
       </c>
-      <c r="G38" s="2" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr">
         <is>
           <t>No loading spinner, progress indicator, or loading message appeared while Admin APIs were deliberately delayed.</t>
         </is>
       </c>
-      <c r="H38" s="2" t="inlineStr">
+      <c r="I38" s="2" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
       </c>
-      <c r="I38" s="2" t="inlineStr">
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>Google Chrome 151 / Windows 11</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
         <is>
           <t>BUG-018</t>
         </is>
       </c>
-      <c r="J38" s="2" t="inlineStr">
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M38" s="2" t="inlineStr">
         <is>
           <t>Async loading state verified.</t>
         </is>
       </c>
-      <c r="K38" s="2" t="inlineStr">
+      <c r="N38" s="2" t="inlineStr">
         <is>
           <t>Executed twice on Google Chrome 151 / Windows. The interface renders empty/default content during data retrieval.</t>
         </is>
       </c>
-      <c r="L38" s="2" t="inlineStr">
+      <c r="O38" s="2" t="inlineStr">
         <is>
           <t>bugs/evidence_images/bug_018_admin_missing_loading_indicator.png</t>
         </is>
@@ -2743,45 +3316,60 @@
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
+          <t>Mobile Product Detail</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
           <t>Check Mobile Product Detail image display and aspect ratio</t>
         </is>
       </c>
-      <c r="E39" s="2" t="inlineStr">
+      <c r="F39" s="2" t="inlineStr">
         <is>
           <t>Mobile Product Detail screen</t>
         </is>
       </c>
-      <c r="F39" s="2" t="inlineStr">
+      <c r="G39" s="2" t="inlineStr">
         <is>
           <t>Product image scales proportionally with aspect ratio preserved (resizeMode='contain')</t>
         </is>
       </c>
-      <c r="G39" s="2" t="inlineStr">
+      <c r="H39" s="2" t="inlineStr">
         <is>
           <t>Not executed on a qualifying mobile environment.</t>
         </is>
       </c>
-      <c r="H39" s="3" t="inlineStr">
+      <c r="I39" s="3" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="I39" s="2" t="inlineStr">
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>Qualifying real mobile device or approved cloud device — pending execution</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J39" s="2" t="inlineStr">
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
         <is>
           <t>Visual image resize mode inspected.</t>
         </is>
       </c>
-      <c r="K39" s="2" t="inlineStr">
+      <c r="N39" s="2" t="inlineStr">
         <is>
           <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
         </is>
       </c>
-      <c r="L39" s="2" t="inlineStr"/>
+      <c r="O39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2801,45 +3389,60 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
+          <t>Mobile Product Detail</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
           <t>Verify product category name display on Mobile Product Detail screen</t>
         </is>
       </c>
-      <c r="E40" s="2" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr">
         <is>
           <t>Product detail screen open</t>
         </is>
       </c>
-      <c r="F40" s="2" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>Product category name displayed below product title</t>
         </is>
       </c>
-      <c r="G40" s="2" t="inlineStr">
+      <c r="H40" s="2" t="inlineStr">
         <is>
           <t>Not executed on a qualifying mobile environment.</t>
         </is>
       </c>
-      <c r="H40" s="3" t="inlineStr">
+      <c r="I40" s="3" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="I40" s="2" t="inlineStr">
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>Qualifying real mobile device or approved cloud device — pending execution</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J40" s="2" t="inlineStr">
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr">
         <is>
           <t>AI missed missing UI element because data was present in backend API JSON; static check failed to detect missing JSX rendering component for category name.</t>
         </is>
       </c>
-      <c r="K40" s="2" t="inlineStr">
+      <c r="N40" s="2" t="inlineStr">
         <is>
           <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
         </is>
       </c>
-      <c r="L40" s="2" t="inlineStr"/>
+      <c r="O40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2859,45 +3462,60 @@
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
+          <t>Mobile Product Detail</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
           <t>Check Mobile Product Detail quantity numeric input field</t>
         </is>
       </c>
-      <c r="E41" s="2" t="inlineStr">
+      <c r="F41" s="2" t="inlineStr">
         <is>
           <t>Product detail screen</t>
         </is>
       </c>
-      <c r="F41" s="2" t="inlineStr">
+      <c r="G41" s="2" t="inlineStr">
         <is>
           <t>Quantity field allows entering numeric values with default 1</t>
         </is>
       </c>
-      <c r="G41" s="2" t="inlineStr">
+      <c r="H41" s="2" t="inlineStr">
         <is>
           <t>Not executed on a qualifying mobile environment.</t>
         </is>
       </c>
-      <c r="H41" s="3" t="inlineStr">
+      <c r="I41" s="3" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="I41" s="2" t="inlineStr">
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>Qualifying real mobile device or approved cloud device — pending execution</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J41" s="2" t="inlineStr">
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr">
         <is>
           <t>Quantity input field binding verified.</t>
         </is>
       </c>
-      <c r="K41" s="2" t="inlineStr">
+      <c r="N41" s="2" t="inlineStr">
         <is>
           <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
         </is>
       </c>
-      <c r="L41" s="2" t="inlineStr"/>
+      <c r="O41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -2917,45 +3535,60 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
+          <t>Mobile Product Detail</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
           <t>Verify Mobile quantity normalization fallback when input is empty or invalid</t>
         </is>
       </c>
-      <c r="E42" s="2" t="inlineStr">
+      <c r="F42" s="2" t="inlineStr">
         <is>
           <t>Empty or non-numeric input</t>
         </is>
       </c>
-      <c r="F42" s="2" t="inlineStr">
+      <c r="G42" s="2" t="inlineStr">
         <is>
           <t>normalizeQuantity coerces invalid input to default 1</t>
         </is>
       </c>
-      <c r="G42" s="2" t="inlineStr">
+      <c r="H42" s="2" t="inlineStr">
         <is>
           <t>Not executed on a qualifying mobile environment.</t>
         </is>
       </c>
-      <c r="H42" s="3" t="inlineStr">
+      <c r="I42" s="3" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="I42" s="2" t="inlineStr">
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>Qualifying real mobile device or approved cloud device — pending execution</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J42" s="2" t="inlineStr">
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr">
         <is>
           <t>Defensive normalization handler verified.</t>
         </is>
       </c>
-      <c r="K42" s="2" t="inlineStr">
+      <c r="N42" s="2" t="inlineStr">
         <is>
           <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
         </is>
       </c>
-      <c r="L42" s="2" t="inlineStr"/>
+      <c r="O42" s="2" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -2975,45 +3608,60 @@
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
+          <t>Mobile Product Detail</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
           <t>Check Mobile Product Detail header back button and home navigation</t>
         </is>
       </c>
-      <c r="E43" s="2" t="inlineStr">
+      <c r="F43" s="2" t="inlineStr">
         <is>
           <t>Product detail screen</t>
         </is>
       </c>
-      <c r="F43" s="2" t="inlineStr">
+      <c r="G43" s="2" t="inlineStr">
         <is>
           <t>Header back button returns user to Product Grid on Home screen</t>
         </is>
       </c>
-      <c r="G43" s="2" t="inlineStr">
+      <c r="H43" s="2" t="inlineStr">
         <is>
           <t>Not executed on a qualifying mobile environment.</t>
         </is>
       </c>
-      <c r="H43" s="3" t="inlineStr">
+      <c r="I43" s="3" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="I43" s="2" t="inlineStr">
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>Qualifying real mobile device or approved cloud device — pending execution</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J43" s="2" t="inlineStr">
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M43" s="2" t="inlineStr">
         <is>
           <t>Navigation stack back action verified.</t>
         </is>
       </c>
-      <c r="K43" s="2" t="inlineStr">
+      <c r="N43" s="2" t="inlineStr">
         <is>
           <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
         </is>
       </c>
-      <c r="L43" s="2" t="inlineStr"/>
+      <c r="O43" s="2" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3033,45 +3681,60 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
+          <t>Mobile Product Detail</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
           <t>Check Mobile 'Thêm vào giỏ hàng' button feedback animation/label state</t>
         </is>
       </c>
-      <c r="E44" s="2" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
         <is>
           <t>Tap 'Thêm vào giỏ hàng'</t>
         </is>
       </c>
-      <c r="F44" s="2" t="inlineStr">
+      <c r="G44" s="2" t="inlineStr">
         <is>
           <t>Button label changes to 'Đã thêm' for 2 seconds then reverts to 'Thêm vào giỏ hàng'</t>
         </is>
       </c>
-      <c r="G44" s="2" t="inlineStr">
+      <c r="H44" s="2" t="inlineStr">
         <is>
           <t>Not executed on a qualifying mobile environment.</t>
         </is>
       </c>
-      <c r="H44" s="3" t="inlineStr">
+      <c r="I44" s="3" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="I44" s="2" t="inlineStr">
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>Qualifying real mobile device or approved cloud device — pending execution</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J44" s="2" t="inlineStr">
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M44" s="2" t="inlineStr">
         <is>
           <t>Temporary state feedback handler verified.</t>
         </is>
       </c>
-      <c r="K44" s="2" t="inlineStr">
+      <c r="N44" s="2" t="inlineStr">
         <is>
           <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
         </is>
       </c>
-      <c r="L44" s="2" t="inlineStr"/>
+      <c r="O44" s="2" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3091,45 +3754,60 @@
       </c>
       <c r="D45" s="2" t="inlineStr">
         <is>
+          <t>Mobile Product Detail</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
           <t>Verify error state display when accessing non-existent Product ID (e.g. /products/999999)</t>
         </is>
       </c>
-      <c r="E45" s="2" t="inlineStr">
+      <c r="F45" s="2" t="inlineStr">
         <is>
           <t>Query non-existent product ID</t>
         </is>
       </c>
-      <c r="F45" s="2" t="inlineStr">
+      <c r="G45" s="2" t="inlineStr">
         <is>
           <t>Renders friendly error component with 'Quay lại trang chủ' CTA navigation button</t>
         </is>
       </c>
-      <c r="G45" s="2" t="inlineStr">
+      <c r="H45" s="2" t="inlineStr">
         <is>
           <t>Not executed on a qualifying mobile environment.</t>
         </is>
       </c>
-      <c r="H45" s="3" t="inlineStr">
+      <c r="I45" s="3" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="I45" s="2" t="inlineStr">
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>Qualifying real mobile device or approved cloud device — pending execution</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J45" s="2" t="inlineStr">
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M45" s="2" t="inlineStr">
         <is>
           <t>AI missed error recovery state gap because API returned HTTP 200 {} instead of 404, misleading UI error handlers into rendering empty fallback text without recovery links.</t>
         </is>
       </c>
-      <c r="K45" s="2" t="inlineStr">
+      <c r="N45" s="2" t="inlineStr">
         <is>
           <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
         </is>
       </c>
-      <c r="L45" s="2" t="inlineStr"/>
+      <c r="O45" s="2" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3149,48 +3827,63 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
+          <t>Mobile Product Detail</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
           <t>Check Mobile Product Detail price display with even vs odd Product IDs</t>
         </is>
       </c>
-      <c r="E46" s="2" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t>Products with string vs number price</t>
         </is>
       </c>
-      <c r="F46" s="2" t="inlineStr">
+      <c r="G46" s="2" t="inlineStr">
         <is>
           <t>Price formatted correctly with toLocaleString() regardless of string/number type</t>
         </is>
       </c>
-      <c r="G46" s="2" t="inlineStr">
+      <c r="H46" s="2" t="inlineStr">
         <is>
           <t>Not executed on a qualifying mobile environment.</t>
         </is>
       </c>
-      <c r="H46" s="3" t="inlineStr">
+      <c r="I46" s="3" t="inlineStr">
         <is>
           <t>Not Executed</t>
         </is>
       </c>
-      <c r="I46" s="2" t="inlineStr">
+      <c r="J46" s="2" t="inlineStr">
+        <is>
+          <t>Qualifying real mobile device or approved cloud device — pending execution</t>
+        </is>
+      </c>
+      <c r="K46" s="2" t="inlineStr">
         <is>
           <t>N/A</t>
         </is>
       </c>
-      <c r="J46" s="2" t="inlineStr">
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>Hybrid</t>
+        </is>
+      </c>
+      <c r="M46" s="2" t="inlineStr">
         <is>
           <t>Number conversion workaround verified.</t>
         </is>
       </c>
-      <c r="K46" s="2" t="inlineStr">
+      <c r="N46" s="2" t="inlineStr">
         <is>
           <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
         </is>
       </c>
-      <c r="L46" s="2" t="inlineStr"/>
+      <c r="O46" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L46"/>
+  <autoFilter ref="A1:O46"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToWidth="1"/>
 </worksheet>

</xml_diff>

<commit_message>
fix(hw03): align mobile checklist with FR-23
</commit_message>
<xml_diff>
--- a/docs/assignments/HW03/deliverables/checklist/gui_checklist.xlsx
+++ b/docs/assignments/HW03/deliverables/checklist/gui_checklist.xlsx
@@ -7,12 +7,14 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GUI Checklist" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Test Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="GUI Checklist" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'GUI Checklist'!$A$1:$O$46</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'GUI Checklist'!$1:$1</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'GUI Checklist'!$A$1:$O$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Summary'!$A$1:$B$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'GUI Checklist'!$A$1:$O$46</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'GUI Checklist'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'GUI Checklist'!$A$1:$O$46</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -34,7 +36,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -48,7 +50,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
+        <fgColor rgb="00E2F0D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -64,7 +71,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -75,6 +82,10 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -438,6 +449,97 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>Measure</t>
+        </is>
+      </c>
+      <c r="B1" s="5" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Designed</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Executed</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Not Executed</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>FR-23 Not Executed</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:B7"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:O46"/>
@@ -451,7 +553,7 @@
     <col width="42" customWidth="1" min="6" max="6"/>
     <col width="42" customWidth="1" min="7" max="7"/>
     <col width="42" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
     <col width="42" customWidth="1" min="10" max="10"/>
     <col width="11" customWidth="1" min="11" max="11"/>
     <col width="11" customWidth="1" min="12" max="12"/>
@@ -578,7 +680,7 @@
           <t>Cart rendered 5 columns (Sản phẩm, Giá, Số lượng, Thành tiền, Thao tác) and displayed the formatted total.</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -651,7 +753,7 @@
           <t>After one click on Product Detail, the cart remained empty; a second click is required.</t>
         </is>
       </c>
-      <c r="I3" s="2" t="inlineStr">
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
@@ -728,7 +830,7 @@
           <t>The product was added with quantity -5 and a negative subtotal (iPhone 15 Pro Max 30.000.000 ₫ -5 -150.000.000 ₫ Xóa).</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr">
+      <c r="I4" s="4" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
@@ -805,7 +907,7 @@
           <t>Entering 2.5 produced cart quantity 2 without any validation message.</t>
         </is>
       </c>
-      <c r="I5" s="2" t="inlineStr">
+      <c r="I5" s="4" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
@@ -882,7 +984,7 @@
           <t>Checkout total is rendered in an editable number input and accepted manual changes.</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr">
+      <c r="I6" s="4" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
@@ -959,7 +1061,7 @@
           <t>Continue shopping links to the product list and the checkout control is available.</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -1032,7 +1134,7 @@
           <t>Unauthenticated checkout displayed “Bạn cần đăng nhập để thanh toán!” and redirected to /login.</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -1105,7 +1207,7 @@
           <t>The empty-cart message and continue-shopping link were displayed after removing the item.</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -1178,7 +1280,7 @@
           <t>The purchased item remained in the cart after checkout completed.</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr">
+      <c r="I10" s="4" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
@@ -1222,7 +1324,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>FR-07</t>
+          <t>FR-23</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1232,37 +1334,37 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Mobile Cart</t>
+          <t>Mobile Product Detail</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Check Mobile Cart layout item row formatting and total sum calculation</t>
+          <t>Verify Mobile Product Detail name, price, description, and overall layout</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Mobile app cart screen</t>
+          <t>A product detail is loaded in the Mobile app</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>ScrollView lists cart items with unit price, quantity edit, item total, and remove button</t>
+          <t>Product name, formatted price, description, and controls are readable and arranged without overlap</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>Not executed on a qualifying mobile environment.</t>
+          <t>Source review found a ScrollView detail card rendering the product image, name, formatted price, description, quantity input, and Add to Cart CTA.</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Qualifying real mobile device or approved cloud device — pending execution</t>
+          <t>Static source review — frontend-mobile/App.js; real-device screenshot pending</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1277,12 +1379,12 @@
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>Mobile React Native component hierarchy correctly analyzed.</t>
+          <t>Source structure supports the required content; physical layout remains subject to screenshot confirmation.</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
+          <t>Source-derived Passed; awaiting real-device confirmation.</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr"/>
@@ -1295,7 +1397,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>FR-07</t>
+          <t>FR-23</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1305,37 +1407,37 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Mobile Cart</t>
+          <t>Mobile Product Detail</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Verify Mobile Cart quantity input change behavior when typing a new number</t>
+          <t>Verify a positive integer quantity is added in the requested amount</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Mobile cart screen</t>
+          <t>Mobile Product Detail is loaded and quantity is a positive integer N</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Typing quantity N sets item quantity to N</t>
+          <t>Tapping Add to Cart adds exactly N units of the selected product</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>Not executed on a qualifying mobile environment.</t>
+          <t>Source review shows a positive integer passes normalizeQuantity unchanged and addToCart stores or adds exactly that quantity.</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Qualifying real mobile device or approved cloud device — pending execution</t>
+          <t>Static source review — frontend-mobile/App.js; real-device screenshot pending</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1350,12 +1452,12 @@
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>AI missed off-by-one arithmetic bug in input change handler because parsed + 1 was misconstrued as an increment button handler rather than direct text input parsing.</t>
+          <t>The addToCart path at lines 129–150 preserves positive integer quantities.</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
+          <t>Source-derived Passed; awaiting real-device confirmation.</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr"/>
@@ -1368,52 +1470,52 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>FR-07</t>
+          <t>FR-23</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>IA-03 Navigation</t>
+          <t>IA-02 Forms &amp; Validation</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Mobile Checkout</t>
+          <t>Mobile Product Detail</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Verify Mobile Checkout payload creation with multi-item cart</t>
+          <t>Verify zero and negative quantities are rejected rather than silently normalized</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Mobile cart with &gt;1 items</t>
+          <t>Mobile Product Detail is loaded</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Full cart array sent in API POST request body</t>
+          <t>Entering 0 or a negative quantity shows validation and does not silently change the value to 1 or add an unintended item</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>Not executed on a qualifying mobile environment.</t>
-        </is>
-      </c>
-      <c r="I13" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>normalizeQuantity returns 1 for zero and negative input; addToCart proceeds and shows a success alert without validation feedback.</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr">
+        <is>
+          <t>Failed</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Qualifying real mobile device or approved cloud device — pending execution</t>
+          <t>Static source review — frontend-mobile/App.js; real-device screenshot pending</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>BUG-022</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
@@ -1423,15 +1525,19 @@
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>AI missed payload array truncation because slice(0, -1) is syntactically clean JavaScript; AI assumed array slicing was used for defensive copying rather than unintended item removal.</t>
+          <t>Boundary source review exposes silent normalization at lines 129–135.</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
-        </is>
-      </c>
-      <c r="O13" s="2" t="inlineStr"/>
+          <t>Source-confirmed defect; runtime screenshot pending.</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>bugs/mobile_source_review.md</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1441,7 +1547,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>FR-07</t>
+          <t>FR-23</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1451,37 +1557,37 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Mobile Cart</t>
+          <t>Mobile Product Detail</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Check Mobile Cart remove item swipe/button confirmation feedback</t>
+          <t>Verify loading state while product details are fetched</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Mobile cart item row</t>
+          <t>Open Mobile Product Detail with a delayed network response</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Clicking 'Xóa' removes item immediately and updates cart badge</t>
+          <t>A visible loading indicator is shown until product data or an error state is available</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>Not executed on a qualifying mobile environment.</t>
+          <t>openProductDetail clears product before fetching; renderProductDetail displays 'Đang tải...' while product is null.</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Qualifying real mobile device or approved cloud device — pending execution</t>
+          <t>Static source review — frontend-mobile/App.js; real-device screenshot pending</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1496,12 +1602,12 @@
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>Mobile array filter state update verified.</t>
+          <t>Loading branch is explicit at lines 114 and 536–542.</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
+          <t>Source-derived Passed; awaiting real-device confirmation.</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr"/>
@@ -1547,7 +1653,7 @@
           <t>A newly created order displayed “Chờ xác nhận” with the pending badge style.</t>
         </is>
       </c>
-      <c r="I15" s="2" t="inlineStr">
+      <c r="I15" s="3" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -1620,7 +1726,7 @@
           <t>The API accepted the valid sequence confirmed → shipping → delivered.</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
+      <c r="I16" s="3" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -1693,7 +1799,7 @@
           <t>The cancellation request returned HTTP 200; the shipping order became canceled.</t>
         </is>
       </c>
-      <c r="I17" s="2" t="inlineStr">
+      <c r="I17" s="4" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
@@ -1770,7 +1876,7 @@
           <t>Canceled → delivered returned HTTP 200; the admin UI displayed the resulting delivered state.</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr">
+      <c r="I18" s="4" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
@@ -1847,7 +1953,7 @@
           <t>SAVE10 (10%) reported savings of -270,000,000 ₫ and a final total of 300,000,000 ₫; the correct values are 3,000,000 ₫ and 27,000,000 ₫.</t>
         </is>
       </c>
-      <c r="I19" s="2" t="inlineStr">
+      <c r="I19" s="4" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
@@ -1924,7 +2030,7 @@
           <t>The invalid coupon displayed the inline message “Mã giảm giá không tồn tại hoặc đã bị vô hiệu hóa”.</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
+      <c r="I20" s="3" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -1997,7 +2103,7 @@
           <t>Checkout displayed a dedicated success state and provided navigation back to the home page.</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
+      <c r="I21" s="3" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -2070,7 +2176,7 @@
           <t>A delivered order rejected a transition back to confirmed with HTTP 400.</t>
         </is>
       </c>
-      <c r="I22" s="2" t="inlineStr">
+      <c r="I22" s="3" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -2143,7 +2249,7 @@
           <t>Order history rendered as a structured five-column table at 1440×1000.</t>
         </is>
       </c>
-      <c r="I23" s="2" t="inlineStr">
+      <c r="I23" s="3" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -2216,7 +2322,7 @@
           <t>Status badges rendered localized labels: Đã hủy, Đã giao, Chờ xác nhận, Chờ xác nhận.</t>
         </is>
       </c>
-      <c r="I24" s="2" t="inlineStr">
+      <c r="I24" s="3" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -2289,7 +2395,7 @@
           <t>The valid Vietnamese number 0912345678 was rejected with “Số điện thoại không hợp lệ. Vui lòng nhập đúng 9-10 chữ số.”.</t>
         </is>
       </c>
-      <c r="I25" s="2" t="inlineStr">
+      <c r="I25" s="4" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
@@ -2366,7 +2472,7 @@
           <t>The address was saved through the profile form; confirmation message: “Cập nhật thành công!”.</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr">
+      <c r="I26" s="3" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -2439,7 +2545,7 @@
           <t>Order-history rows provide no expansion control, details link, or item-level view.</t>
         </is>
       </c>
-      <c r="I27" s="2" t="inlineStr">
+      <c r="I27" s="4" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
@@ -2516,7 +2622,7 @@
           <t>The order-history empty state was displayed for a user with no orders at the start of execution.</t>
         </is>
       </c>
-      <c r="I28" s="2" t="inlineStr">
+      <c r="I28" s="3" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -2556,47 +2662,47 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>FR-11</t>
+          <t>FR-23</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>IA-01 General UI</t>
+          <t>IA-04 Feedback &amp; State</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Mobile Profile</t>
+          <t>Mobile Product Detail</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Check Mobile Profile order cards summary display</t>
+          <t>Verify repeated additions of the same product update quantity consistently</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Mobile Profile screen</t>
+          <t>The same product is already present in the cart</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>ScrollView displays order card with ID, Date, Formatted Amount, and Status</t>
+          <t>Adding the product again updates its quantity consistently without a duplicate or lost update</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>Not executed on a qualifying mobile environment.</t>
+          <t>Source review finds the existing product by ID and replaces that row with old quantity plus the requested safe quantity.</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>Qualifying real mobile device or approved cloud device — pending execution</t>
+          <t>Static source review — frontend-mobile/App.js; real-device screenshot pending</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
@@ -2611,12 +2717,12 @@
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>Mobile React Native component verified.</t>
+          <t>Existing-item update is implemented at lines 136–148 without creating a duplicate row.</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
+          <t>Source-derived Passed; awaiting real-device confirmation.</t>
         </is>
       </c>
       <c r="O29" s="2" t="inlineStr"/>
@@ -2629,47 +2735,47 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>FR-11</t>
+          <t>FR-23</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>IA-04 Feedback &amp; State</t>
+          <t>IA-01 General UI</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Mobile Profile</t>
+          <t>Mobile Product Detail</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Check Web vs Mobile 'Hủy đơn' button visibility inconsistency</t>
+          <t>Verify content and primary CTA remain visible on a small screen</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Order in shipping state viewed on Mobile vs Web</t>
+          <t>Mobile Product Detail is opened on the smallest qualifying device viewport</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Button visibility consistent across platforms (hidden for shipping)</t>
+          <t>Product content can be read and the Add to Cart CTA can be reached without clipping, overlap, or obstruction</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>Not executed on a qualifying mobile environment.</t>
+          <t>Source review places the full detail card and CTA inside a vertical ScrollView with padded responsive width.</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>Qualifying real mobile device or approved cloud device — pending execution</t>
+          <t>Static source review — frontend-mobile/App.js; real-device screenshot pending</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
@@ -2684,12 +2790,12 @@
       </c>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>UI rendering discrepancy noted between web profile and mobile profile.</t>
+          <t>ScrollView makes the CTA reachable in the source layout; clipping must be rechecked from the smallest-device screenshot.</t>
         </is>
       </c>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>The Web behavior was inspected, but the comparison requires execution of the Mobile app.</t>
+          <t>Source-derived Passed; awaiting real-device confirmation.</t>
         </is>
       </c>
       <c r="O30" s="2" t="inlineStr"/>
@@ -2735,7 +2841,7 @@
           <t>Dashboard displayed revenue and order-count summary cards.</t>
         </is>
       </c>
-      <c r="I31" s="2" t="inlineStr">
+      <c r="I31" s="3" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -2808,7 +2914,7 @@
           <t>Delivered-order revenue should total 8,234,567 ₫; the dashboard rendered Tổng doanh thu (Delivered) 16.469.134 ₫.</t>
         </is>
       </c>
-      <c r="I32" s="2" t="inlineStr">
+      <c r="I32" s="4" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
@@ -2885,7 +2991,7 @@
           <t>Stored shipping-address HTML was interpreted as markup in the Admin Orders table.</t>
         </is>
       </c>
-      <c r="I33" s="2" t="inlineStr">
+      <c r="I33" s="4" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
@@ -2962,7 +3068,7 @@
           <t>The pending order exposed the expected actions: Xác nhận, Hủy.</t>
         </is>
       </c>
-      <c r="I34" s="2" t="inlineStr">
+      <c r="I34" s="3" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -3035,7 +3141,7 @@
           <t>All six primary admin navigation destinations were visible and selectable.</t>
         </is>
       </c>
-      <c r="I35" s="2" t="inlineStr">
+      <c r="I35" s="3" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -3108,7 +3214,7 @@
           <t>The status changed to Đã xác nhận, but no success toast or confirmation message appeared.</t>
         </is>
       </c>
-      <c r="I36" s="2" t="inlineStr">
+      <c r="I36" s="4" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
@@ -3185,7 +3291,7 @@
           <t>Editing one product changed every visible product name in client state.</t>
         </is>
       </c>
-      <c r="I37" s="2" t="inlineStr">
+      <c r="I37" s="4" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
@@ -3262,7 +3368,7 @@
           <t>No loading spinner, progress indicator, or loading message appeared while Admin APIs were deliberately delayed.</t>
         </is>
       </c>
-      <c r="I38" s="2" t="inlineStr">
+      <c r="I38" s="4" t="inlineStr">
         <is>
           <t>Failed</t>
         </is>
@@ -3306,7 +3412,7 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>Pool D</t>
+          <t>FR-23</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -3336,22 +3442,22 @@
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>Not executed on a qualifying mobile environment.</t>
-        </is>
-      </c>
-      <c r="I39" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>The Product Detail Image explicitly uses resizeMode='stretch', which forces content into a fixed 100%-by-240 layout and does not preserve aspect ratio.</t>
+        </is>
+      </c>
+      <c r="I39" s="4" t="inlineStr">
+        <is>
+          <t>Failed</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>Qualifying real mobile device or approved cloud device — pending execution</t>
+          <t>Static source review — frontend-mobile/App.js; real-device screenshot pending</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>BUG-020</t>
         </is>
       </c>
       <c r="L39" s="2" t="inlineStr">
@@ -3361,15 +3467,19 @@
       </c>
       <c r="M39" s="2" t="inlineStr">
         <is>
-          <t>Visual image resize mode inspected.</t>
+          <t>The conflicting resize mode is explicit at App.js line 558.</t>
         </is>
       </c>
       <c r="N39" s="2" t="inlineStr">
         <is>
-          <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
-        </is>
-      </c>
-      <c r="O39" s="2" t="inlineStr"/>
+          <t>Source-confirmed defect; runtime screenshot pending.</t>
+        </is>
+      </c>
+      <c r="O39" s="2" t="inlineStr">
+        <is>
+          <t>bugs/mobile_source_review.md</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3379,7 +3489,7 @@
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>Pool D</t>
+          <t>FR-23</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -3409,22 +3519,22 @@
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>Not executed on a qualifying mobile environment.</t>
-        </is>
-      </c>
-      <c r="I40" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>The Product Detail JSX renders name, price, and description but contains no category field or category label.</t>
+        </is>
+      </c>
+      <c r="I40" s="4" t="inlineStr">
+        <is>
+          <t>Failed</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>Qualifying real mobile device or approved cloud device — pending execution</t>
+          <t>Static source review — frontend-mobile/App.js; real-device screenshot pending</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>BUG-021</t>
         </is>
       </c>
       <c r="L40" s="2" t="inlineStr">
@@ -3434,15 +3544,19 @@
       </c>
       <c r="M40" s="2" t="inlineStr">
         <is>
-          <t>AI missed missing UI element because data was present in backend API JSON; static check failed to detect missing JSX rendering component for category name.</t>
+          <t>The render block at lines 560–562 omits category even when product data contains it.</t>
         </is>
       </c>
       <c r="N40" s="2" t="inlineStr">
         <is>
-          <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
-        </is>
-      </c>
-      <c r="O40" s="2" t="inlineStr"/>
+          <t>Source-confirmed defect; runtime screenshot pending.</t>
+        </is>
+      </c>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>bugs/mobile_source_review.md</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3452,7 +3566,7 @@
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>Pool D</t>
+          <t>FR-23</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -3482,17 +3596,17 @@
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>Not executed on a qualifying mobile environment.</t>
+          <t>Source review initializes quantity to '1' and binds it to a TextInput configured with keyboardType='numeric'.</t>
         </is>
       </c>
       <c r="I41" s="3" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>Qualifying real mobile device or approved cloud device — pending execution</t>
+          <t>Static source review — frontend-mobile/App.js; real-device screenshot pending</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr">
@@ -3507,12 +3621,12 @@
       </c>
       <c r="M41" s="2" t="inlineStr">
         <is>
-          <t>Quantity input field binding verified.</t>
+          <t>Default value and numeric keyboard binding are explicit in the component.</t>
         </is>
       </c>
       <c r="N41" s="2" t="inlineStr">
         <is>
-          <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
+          <t>Source-derived Passed; awaiting real-device confirmation.</t>
         </is>
       </c>
       <c r="O41" s="2" t="inlineStr"/>
@@ -3525,7 +3639,7 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>Pool D</t>
+          <t>FR-23</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -3540,7 +3654,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Verify Mobile quantity normalization fallback when input is empty or invalid</t>
+          <t>Verify invalid or empty quantity receives validation feedback</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -3550,27 +3664,27 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>normalizeQuantity coerces invalid input to default 1</t>
+          <t>The app rejects invalid input, explains the problem, and does not add an unintended quantity</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>Not executed on a qualifying mobile environment.</t>
-        </is>
-      </c>
-      <c r="I42" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>normalizeQuantity coerces empty or non-numeric input to 1; addToCart continues and reports success instead of validation feedback.</t>
+        </is>
+      </c>
+      <c r="I42" s="4" t="inlineStr">
+        <is>
+          <t>Failed</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
         <is>
-          <t>Qualifying real mobile device or approved cloud device — pending execution</t>
+          <t>Static source review — frontend-mobile/App.js; real-device screenshot pending</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>BUG-022</t>
         </is>
       </c>
       <c r="L42" s="2" t="inlineStr">
@@ -3580,15 +3694,19 @@
       </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
-          <t>Defensive normalization handler verified.</t>
+          <t>The original fallback expectation was corrected to the user-facing validation oracle; lines 129–135 silently normalize invalid input.</t>
         </is>
       </c>
       <c r="N42" s="2" t="inlineStr">
         <is>
-          <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
-        </is>
-      </c>
-      <c r="O42" s="2" t="inlineStr"/>
+          <t>Source-confirmed defect shared with CHK-GUI-012; runtime screenshot pending.</t>
+        </is>
+      </c>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>bugs/mobile_source_review.md</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3598,7 +3716,7 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>Pool D</t>
+          <t>FR-23</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -3628,22 +3746,22 @@
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>Not executed on a qualifying mobile environment.</t>
-        </is>
-      </c>
-      <c r="I43" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>The shared header provides a tappable EShop Mobile brand that calls goHome, but Product Detail renders no dedicated back control as required by this check.</t>
+        </is>
+      </c>
+      <c r="I43" s="4" t="inlineStr">
+        <is>
+          <t>Failed</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
-          <t>Qualifying real mobile device or approved cloud device — pending execution</t>
+          <t>Static source review — frontend-mobile/App.js; real-device screenshot pending</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>BUG-023</t>
         </is>
       </c>
       <c r="L43" s="2" t="inlineStr">
@@ -3653,15 +3771,19 @@
       </c>
       <c r="M43" s="2" t="inlineStr">
         <is>
-          <t>Navigation stack back action verified.</t>
+          <t>Navigation to home exists only through the brand; the Product Detail render block has no back button.</t>
         </is>
       </c>
       <c r="N43" s="2" t="inlineStr">
         <is>
-          <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
-        </is>
-      </c>
-      <c r="O43" s="2" t="inlineStr"/>
+          <t>Source-confirmed defect; runtime screenshot pending.</t>
+        </is>
+      </c>
+      <c r="O43" s="2" t="inlineStr">
+        <is>
+          <t>bugs/mobile_source_review.md</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3671,7 +3793,7 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>Pool D</t>
+          <t>FR-23</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -3701,17 +3823,17 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>Not executed on a qualifying mobile environment.</t>
+          <t>The add handler sets added=true, renders 'Đã thêm', and schedules setAdded(false) after 2000 ms; addToCart also raises a success Alert.</t>
         </is>
       </c>
       <c r="I44" s="3" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="J44" s="2" t="inlineStr">
         <is>
-          <t>Qualifying real mobile device or approved cloud device — pending execution</t>
+          <t>Static source review — frontend-mobile/App.js; real-device screenshot pending</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
@@ -3726,12 +3848,12 @@
       </c>
       <c r="M44" s="2" t="inlineStr">
         <is>
-          <t>Temporary state feedback handler verified.</t>
+          <t>Temporary feedback is explicit at lines 575–583.</t>
         </is>
       </c>
       <c r="N44" s="2" t="inlineStr">
         <is>
-          <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
+          <t>Source-derived Passed; awaiting real-device confirmation.</t>
         </is>
       </c>
       <c r="O44" s="2" t="inlineStr"/>
@@ -3744,7 +3866,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>Pool D</t>
+          <t>FR-23</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -3774,22 +3896,22 @@
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>Not executed on a qualifying mobile environment.</t>
-        </is>
-      </c>
-      <c r="I45" s="3" t="inlineStr">
-        <is>
-          <t>Not Executed</t>
+          <t>An empty product renders technical text describing a blank-page error and provides no recovery CTA or navigation control in the error body.</t>
+        </is>
+      </c>
+      <c r="I45" s="4" t="inlineStr">
+        <is>
+          <t>Failed</t>
         </is>
       </c>
       <c r="J45" s="2" t="inlineStr">
         <is>
-          <t>Qualifying real mobile device or approved cloud device — pending execution</t>
+          <t>Static source review — frontend-mobile/App.js; real-device screenshot pending</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>BUG-024</t>
         </is>
       </c>
       <c r="L45" s="2" t="inlineStr">
@@ -3799,15 +3921,19 @@
       </c>
       <c r="M45" s="2" t="inlineStr">
         <is>
-          <t>AI missed error recovery state gap because API returned HTTP 200 {} instead of 404, misleading UI error handlers into rendering empty fallback text without recovery links.</t>
+          <t>The empty-object branch at lines 544–550 lacks the expected recovery action.</t>
         </is>
       </c>
       <c r="N45" s="2" t="inlineStr">
         <is>
-          <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
-        </is>
-      </c>
-      <c r="O45" s="2" t="inlineStr"/>
+          <t>Source-confirmed defect; runtime screenshot pending.</t>
+        </is>
+      </c>
+      <c r="O45" s="2" t="inlineStr">
+        <is>
+          <t>bugs/mobile_source_review.md</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3817,7 +3943,7 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>Pool D</t>
+          <t>FR-23</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -3847,17 +3973,17 @@
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>Not executed on a qualifying mobile environment.</t>
+          <t>formatMoney converts every value with Number(value) before applying toLocaleString, covering numeric and numeric-string prices.</t>
         </is>
       </c>
       <c r="I46" s="3" t="inlineStr">
         <is>
-          <t>Not Executed</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
-          <t>Qualifying real mobile device or approved cloud device — pending execution</t>
+          <t>Static source review — frontend-mobile/App.js; real-device screenshot pending</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -3872,12 +3998,12 @@
       </c>
       <c r="M46" s="2" t="inlineStr">
         <is>
-          <t>Number conversion workaround verified.</t>
+          <t>The conversion is explicit in formatMoney near the top of App.js.</t>
         </is>
       </c>
       <c r="N46" s="2" t="inlineStr">
         <is>
-          <t>Requires Expo Go on a physical device or an approved cloud-device platform.</t>
+          <t>Source-derived Passed; awaiting real-device confirmation.</t>
         </is>
       </c>
       <c r="O46" s="2" t="inlineStr"/>

</xml_diff>